<commit_message>
docs: horarios por curso (ES 8h30-10h10, SI 10h20-12h00) e aula 2 = intro Python/Colab
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VMrx4Ermpivez1KA1szDim
</commit_message>
<xml_diff>
--- a/docs/PID - Bases de Sistema de Informação 3 - Estatística e Probabilidade - 2.2026.xlsx
+++ b/docs/PID - Bases de Sistema de Informação 3 - Estatística e Probabilidade - 2.2026.xlsx
@@ -891,7 +891,7 @@
       </c>
       <c r="B4" s="49" t="inlineStr">
         <is>
-          <t>Sistemas de Informação</t>
+          <t>Engenharia de Software e Sistemas de Informação</t>
         </is>
       </c>
       <c r="C4" s="50" t="n"/>
@@ -987,7 +987,7 @@
       </c>
       <c r="B7" s="49" t="inlineStr">
         <is>
-          <t>Bases de Sistema de Informação 3 — Estatística e Probabilidade — 40 horas. Encontros semanais às sextas-feiras, das 10h45 às 12h45. Ementa: estatística aplicada para quem constrói software e trabalha com dados — análise exploratória de dados; probabilidade e distribuições; amostragem, distribuições amostrais e estimação; testes de significância (testes A/B, testes de hipótese, valores-p e testes t); e regressão e predição. Exemplos em Python.</t>
+          <t>Bases de Sistema de Informação 3 — Estatística e Probabilidade — 40 horas. Encontros semanais às sextas-feiras: Engenharia de Software das 8h30 às 10h10; Sistemas de Informação das 10h20 às 12h00. Ementa: estatística aplicada para quem constrói software e trabalha com dados — análise exploratória de dados; probabilidade e distribuições; amostragem, distribuições amostrais e estimação; testes de significância (testes A/B, testes de hipótese, valores-p e testes t); e regressão e predição. Exemplos em Python.</t>
         </is>
       </c>
       <c r="C7" s="50" t="n"/>
@@ -1282,7 +1282,7 @@
       </c>
       <c r="C24" s="80" t="inlineStr">
         <is>
-          <t>Capítulo 1 — Análise Exploratória de Dados: elementos de dados estruturados e dados retangulares; estimativas de localização (média, média aparada, mediana, moda, ponderadas).</t>
+          <t>Introdução ao Python e ao Google Colab: o ambiente de execução dos exemplos da disciplina; noções básicas da linguagem para acompanhar o código.</t>
         </is>
       </c>
       <c r="D24" s="59" t="n"/>
@@ -1298,7 +1298,7 @@
       </c>
       <c r="C25" s="80" t="inlineStr">
         <is>
-          <t>Capítulo 1 — Estimativas de variabilidade: variância, desvio-padrão, IQR, MAD e escores-padrão (z-scores).</t>
+          <t>Capítulo 1 — Análise Exploratória de Dados: elementos de dados estruturados e dados retangulares; estimativas de localização (média, média aparada, mediana, moda, ponderadas).</t>
         </is>
       </c>
       <c r="D25" s="59" t="n"/>
@@ -1314,7 +1314,7 @@
       </c>
       <c r="C26" s="80" t="inlineStr">
         <is>
-          <t>Capítulo 1 — Explorando a distribuição dos dados: percentis, boxplot, histograma, densidade, assimetria, curtose e gráfico de violino.</t>
+          <t>Capítulo 1 — Estimativas de variabilidade (variância, desvio-padrão, IQR, MAD, escores-padrão); explorando a distribuição dos dados (percentis, boxplot, histograma, densidade, assimetria, curtose, violino).</t>
         </is>
       </c>
       <c r="D26" s="59" t="n"/>

</xml_diff>

<commit_message>
docs: PID — conteudo do cap2 no cronograma (condicional/bayes, contagem, hipergeometrica)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01SJaYmn8DhrwsSNaPLehpcV
</commit_message>
<xml_diff>
--- a/docs/PID - Bases de Sistema de Informação 3 - Estatística e Probabilidade - 2.2026.xlsx
+++ b/docs/PID - Bases de Sistema de Informação 3 - Estatística e Probabilidade - 2.2026.xlsx
@@ -1346,7 +1346,7 @@
       </c>
       <c r="C28" s="80" t="inlineStr">
         <is>
-          <t>Capítulo 2 — Probabilidade e Distribuições: o que é probabilidade (frequentista e bayesiana) e regras de probabilidade; distribuição binomial; distribuição de Poisson.</t>
+          <t>Capítulo 2 — Probabilidade e Distribuições: o que é probabilidade; regras de probabilidade; probabilidade condicional e Teorema de Bayes.</t>
         </is>
       </c>
       <c r="D28" s="59" t="n"/>
@@ -1362,7 +1362,7 @@
       </c>
       <c r="C29" s="80" t="inlineStr">
         <is>
-          <t>Capítulo 2 — Distribuição normal; distribuições de cauda longa; distribuição t de Student.</t>
+          <t>Capítulo 2 — Contagem (permutação e combinação); distribuição binomial; distribuição hipergeométrica.</t>
         </is>
       </c>
       <c r="D29" s="59" t="n"/>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="C30" s="80" t="inlineStr">
         <is>
-          <t>Capítulo 2 — Distribuição qui-quadrado; distribuição F. Revisão para a Prova 1.</t>
+          <t>Capítulo 2 — Distribuição normal; distribuições de cauda longa. Revisão para a Prova 1.</t>
         </is>
       </c>
       <c r="D30" s="59" t="n"/>

</xml_diff>